<commit_message>
update session 3 paper order
</commit_message>
<xml_diff>
--- a/2026/FMSys'26 Program.xlsx
+++ b/2026/FMSys'26 Program.xlsx
@@ -930,12 +930,12 @@
       <c r="B22" s="12" t="n"/>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>X-CPS: A Top-Down Hierarchical Framework for Explaining Learning-enabled Cyber-Physical Systems</t>
+          <t>Characterizing Cellular Network Dynamics for Federated Human Activity Recognition</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Guocheng He, Lingwen Deng, Ziyan An, Meiyi Ma (Vanderbilt University)</t>
+          <t>Muhammad Abdullah Soomro, Muhammad Shayan Nazeer, Taqi Raza, Fatima Anwar (University of Massachusetts Amherst)</t>
         </is>
       </c>
     </row>
@@ -944,12 +944,12 @@
       <c r="B23" s="12" t="n"/>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Characterizing Cellular Network Dynamics for Federated Human Activity Recognition</t>
+          <t>X-CPS: A Top-Down Hierarchical Framework for Explaining Learning-enabled Cyber-Physical Systems</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Muhammad Abdullah Soomro, Muhammad Shayan Nazeer, Taqi Raza, Fatima Anwar (University of Massachusetts Amherst)</t>
+          <t>Guocheng He, Lingwen Deng, Ziyan An, Meiyi Ma (Vanderbilt University)</t>
         </is>
       </c>
     </row>

</xml_diff>